<commit_message>
Add binary search problems, SRS session files, and handoff doc
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Python/Leetcode Log.xlsx
+++ b/Python/Leetcode Log.xlsx
@@ -2429,7 +2429,7 @@
         </is>
       </c>
       <c r="B96" s="22" t="n">
-        <v>46166.4290880051</v>
+        <v>46166.42908800926</v>
       </c>
       <c r="C96" s="0" t="inlineStr">
         <is>
@@ -2459,7 +2459,7 @@
         </is>
       </c>
       <c r="B97" s="22" t="n">
-        <v>46166.4290880051</v>
+        <v>46166.42908800926</v>
       </c>
       <c r="C97" s="0" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add binary search SRS file, update two pointers SRS and Leetcode Log
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Python/Leetcode Log.xlsx
+++ b/Python/Leetcode Log.xlsx
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="B18" s="17" t="n">
-        <v>45889</v>
+        <v>46183</v>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="B19" s="17" t="n">
-        <v>45889</v>
+        <v>46183</v>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>

</xml_diff>